<commit_message>
added strict incremental ordering to rule logic but to check validation results further
</commit_message>
<xml_diff>
--- a/rules/CORE-000535/negative/01/data/unit-test-coreid-CG0620-negative 1.xlsx
+++ b/rules/CORE-000535/negative/01/data/unit-test-coreid-CG0620-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000535\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB091DD-CD18-499F-BC20-253E39AB2AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40562809-E9A4-4A7F-A09D-84C01D1CD8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="4" xr2:uid="{68203D44-07AE-4443-B366-E6DFDE0510A4}"/>
+    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{68203D44-07AE-4443-B366-E6DFDE0510A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="79">
   <si>
     <t>Product</t>
   </si>
@@ -439,7 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -487,9 +487,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -958,7 +955,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BEEBCD-2776-477F-B12E-85A72C199137}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="12.28515625" customWidth="1"/>
@@ -1100,7 +1097,7 @@
       <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1195,13 +1192,13 @@
         <v>78</v>
       </c>
       <c r="D12">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
         <v>43</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1215,13 +1212,13 @@
         <v>78</v>
       </c>
       <c r="D13">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" t="s">
         <v>46</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1235,13 +1232,13 @@
         <v>78</v>
       </c>
       <c r="D14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E14" t="s">
         <v>43</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1255,13 +1252,13 @@
         <v>78</v>
       </c>
       <c r="D15">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1275,13 +1272,13 @@
         <v>78</v>
       </c>
       <c r="D16">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E16" t="s">
         <v>43</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1295,12 +1292,52 @@
         <v>78</v>
       </c>
       <c r="D17">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E17" t="s">
         <v>46</v>
       </c>
       <c r="F17" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>9</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1774,8 +1811,8 @@
       <c r="C8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="12">
-        <v>4</v>
+      <c r="D8" s="13">
+        <v>5</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>64</v>
@@ -1783,7 +1820,7 @@
       <c r="F8" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="14" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>